<commit_message>
Suppression de proposition modifiee 7c24249e398b587e37ea21b6a7221a800847e998
</commit_message>
<xml_diff>
--- a/AnalysePharma/ig/CodeSystem-fr-pharmaceutical-intervention-devenir-code.xlsx
+++ b/AnalysePharma/ig/CodeSystem-fr-pharmaceutical-intervention-devenir-code.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="43">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-04-14T15:34:16+00:00</t>
+    <t>2026-04-30T09:49:26+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -120,7 +120,7 @@
     <t>Count</t>
   </si>
   <si>
-    <t>4</t>
+    <t>2</t>
   </si>
   <si>
     <t>Level</t>
@@ -141,19 +141,7 @@
     <t>Acceptée</t>
   </si>
   <si>
-    <t>2</t>
-  </si>
-  <si>
     <t>Non-acceptée</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>Non renseigné</t>
-  </si>
-  <si>
-    <t>Acceptée avec modification de proposition(s)</t>
   </si>
 </sst>
 </file>
@@ -461,7 +449,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -495,36 +483,12 @@
         <v>40</v>
       </c>
       <c r="B3" t="s" s="2">
+        <v>35</v>
+      </c>
+      <c r="C3" t="s" s="2">
         <v>42</v>
       </c>
-      <c r="C3" t="s" s="2">
-        <v>43</v>
-      </c>
       <c r="D3" s="2"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="s" s="2">
-        <v>40</v>
-      </c>
-      <c r="B4" t="s" s="2">
-        <v>44</v>
-      </c>
-      <c r="C4" t="s" s="2">
-        <v>45</v>
-      </c>
-      <c r="D4" s="2"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="s" s="2">
-        <v>40</v>
-      </c>
-      <c r="B5" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="C5" t="s" s="2">
-        <v>46</v>
-      </c>
-      <c r="D5" s="2"/>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>

</xml_diff>